<commit_message>
Describe what I changed
</commit_message>
<xml_diff>
--- a/DummyData.xlsx
+++ b/DummyData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mintal\PycharmProjects\pythonProject\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mintal\PycharmProjects\pythonProject\test_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E351B897-9CAA-477F-9F45-FEB6FECB64F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA88966D-410A-400A-B759-CAD5966C1F92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="744" activeTab="2" xr2:uid="{0866BE8F-DC35-4B49-B44D-F3C4BC13F9EF}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="111">
   <si>
     <t>MSID</t>
   </si>
@@ -216,18 +216,6 @@
     <t>Coronary Artery Disease</t>
   </si>
   <si>
-    <t>DB</t>
-  </si>
-  <si>
-    <t>Diabetes</t>
-  </si>
-  <si>
-    <t>BPH</t>
-  </si>
-  <si>
-    <t>Benign Prostatic Hypertrophy</t>
-  </si>
-  <si>
     <t>PHS 2.0</t>
   </si>
   <si>
@@ -276,9 +264,6 @@
     <t>Program ID - 836784495</t>
   </si>
   <si>
-    <t>Display "Member is NOT eligible. Opt Out Preference is set to DNC. Please process reject referral ."</t>
-  </si>
-  <si>
     <t>SCENARIOS</t>
   </si>
   <si>
@@ -291,13 +276,7 @@
     <t>Program ID - 498822475</t>
   </si>
   <si>
-    <t>Display "Member age is below 18 yrs old and is NOT eligible. Please create a GCM referral."</t>
-  </si>
-  <si>
     <t>Program ID - 683294865</t>
-  </si>
-  <si>
-    <t>Display "Member is NOT eligible. Please create a surveillance assignment."</t>
   </si>
   <si>
     <r>
@@ -349,9 +328,6 @@
       <t xml:space="preserve"> 
 Opt out preference = DNC</t>
     </r>
-  </si>
-  <si>
-    <t>Display "Member is NOT eligible. Please reassign to real time work queue ."</t>
   </si>
   <si>
     <t>ABS</t>
@@ -483,9 +459,6 @@
 Program Type is PHS 2.0 or 3.0
 Policy record found in MGRL</t>
     </r>
-  </si>
-  <si>
-    <t>Policy_End_Date</t>
   </si>
   <si>
     <r>
@@ -550,10 +523,62 @@
     </r>
   </si>
   <si>
-    <t>Display "Member is NOT eligible. Please process reject referral."</t>
-  </si>
-  <si>
     <t>Display "Member is NOT eligible. Please reassign the case to the correct work queue."</t>
+  </si>
+  <si>
+    <t>ABC</t>
+  </si>
+  <si>
+    <t>Program ID - 350339412</t>
+  </si>
+  <si>
+    <t>Member_Policy_End_Date</t>
+  </si>
+  <si>
+    <t>Member_Funding_Arrangement</t>
+  </si>
+  <si>
+    <t>Member_Opt_Out_Date</t>
+  </si>
+  <si>
+    <t>Based from the following parameters, Member is NOT eligible:
+Member age is &lt;age&gt;
+Member Program: General Condition Management
+Member case status: Open
+Member discharge date: Not yet discharged
+RECOMMENDED ACTION: Create a surveillance assignment.</t>
+  </si>
+  <si>
+    <t>Based from the following parameters, Member is NOT eligible:
+Member age is  &lt;age&gt;  yrs old
+Member Program: &lt;Program name&gt;
+RECOMMENDED ACTION: Create a GCM referral."</t>
+  </si>
+  <si>
+    <t>Based from the following parameters, Member is NOT eligible:
+Opt Out Preference: DNC
+Member opt out date: mm/dd/yyyy
+RECOMMENDED ACTION: Process reject referral.</t>
+  </si>
+  <si>
+    <t>Based from the following parameters, Member is NOT eligible:
+Age (in yrs) :  &lt;age&gt;
+Program : General Condition Management
+Case status : Close
+Discharge date : &lt;discharged date&gt;
+Program type : &lt;program type&gt;
+RECOMMENDED ACTION : Reassign to real time work queue .</t>
+  </si>
+  <si>
+    <t>Based from the following parameters, Member is NOT eligible:
+Age (in yrs) :  &lt;age&gt;
+Program : General Condition Management
+Case status : Close
+Discharge date : &lt;discharged date&gt;
+Program type : &lt;program type&gt;
+Policy End Date: &lt;policy end date&gt;
+Policy record NOT found in MGRL
+RECOMMENDED ACTION :  Please process reject referral.</t>
   </si>
 </sst>
 </file>
@@ -639,7 +664,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -680,6 +705,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1019,7 +1045,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11DF451D-8CA4-48BE-BE99-8F5EDF1684B2}">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1032,12 +1058,14 @@
     <col min="8" max="8" width="17.7265625" customWidth="1"/>
     <col min="9" max="9" width="15.36328125" customWidth="1"/>
     <col min="10" max="10" width="25.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" customWidth="1"/>
-    <col min="12" max="12" width="27.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.1796875" customWidth="1"/>
+    <col min="12" max="12" width="16.1796875" customWidth="1"/>
+    <col min="13" max="13" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.90625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="26.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -1048,16 +1076,16 @@
         <v>20</v>
       </c>
       <c r="D1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="G1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="H1" t="s">
         <v>29</v>
@@ -1066,19 +1094,25 @@
         <v>47</v>
       </c>
       <c r="J1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="K1" t="s">
+        <v>105</v>
+      </c>
+      <c r="L1" t="s">
+        <v>95</v>
+      </c>
+      <c r="M1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N1" t="s">
         <v>103</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>104</v>
       </c>
-      <c r="M1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>4088042736</v>
       </c>
@@ -1104,14 +1138,14 @@
       <c r="H2">
         <v>376681962</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>708881</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2800672319</v>
       </c>
@@ -1138,16 +1172,19 @@
         <v>836784495</v>
       </c>
       <c r="J3" t="s">
-        <v>74</v>
-      </c>
-      <c r="K3">
+        <v>70</v>
+      </c>
+      <c r="K3" s="1">
+        <v>46296</v>
+      </c>
+      <c r="L3">
         <v>476897</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1125525865</v>
       </c>
@@ -1173,14 +1210,14 @@
       <c r="H4" s="8">
         <v>498822475</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>909166</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>8104375203</v>
       </c>
@@ -1206,14 +1243,14 @@
       <c r="H5">
         <v>133324351</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>982065</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>6724421141</v>
       </c>
@@ -1224,11 +1261,11 @@
         <v>37</v>
       </c>
       <c r="D6" s="1">
-        <v>30014</v>
+        <v>40972</v>
       </c>
       <c r="E6" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="F6" t="s">
         <v>27</v>
@@ -1236,14 +1273,20 @@
       <c r="G6" t="s">
         <v>28</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="20">
         <v>350339412</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>1324</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N6" s="1">
+        <v>2958465</v>
+      </c>
+      <c r="O6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>3428511303</v>
       </c>
@@ -1254,11 +1297,11 @@
         <v>33</v>
       </c>
       <c r="D7" s="1">
-        <v>32603</v>
+        <v>41369</v>
       </c>
       <c r="E7" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="F7" t="s">
         <v>27</v>
@@ -1269,11 +1312,11 @@
       <c r="H7" s="10">
         <v>683294865</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>4678</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7373366639</v>
       </c>
@@ -1284,11 +1327,11 @@
         <v>40</v>
       </c>
       <c r="D8" s="1">
-        <v>34825</v>
+        <v>40304</v>
       </c>
       <c r="E8" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="F8" t="s">
         <v>27</v>
@@ -1299,8 +1342,14 @@
       <c r="H8" s="18">
         <v>543531255</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="L8">
+        <v>457698</v>
+      </c>
+      <c r="N8" s="1">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>6350095935</v>
       </c>
@@ -1326,11 +1375,11 @@
       <c r="H9" s="12">
         <v>344284704</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>469657</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>3141284892</v>
       </c>
@@ -1356,7 +1405,7 @@
       <c r="H10" s="14">
         <v>435328172</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>145344</v>
       </c>
     </row>
@@ -1381,10 +1430,10 @@
         <v>19</v>
       </c>
       <c r="B1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D1" t="s">
         <v>45</v>
@@ -1451,10 +1500,10 @@
         <v>350339412</v>
       </c>
       <c r="B6" t="s">
-        <v>56</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
         <v>46</v>
@@ -1479,10 +1528,10 @@
         <v>543531255</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
         <v>46</v>
@@ -1499,7 +1548,7 @@
         <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -1513,7 +1562,7 @@
         <v>15</v>
       </c>
       <c r="D10" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1535,88 +1584,90 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="58" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>85</v>
-      </c>
       <c r="B2" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="87" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="87" x14ac:dyDescent="0.35">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="B8" s="19"/>
+        <v>99</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>102</v>
+      </c>
       <c r="C8" s="4" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1636,16 +1687,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -1653,7 +1704,7 @@
         <v>4088042736</v>
       </c>
       <c r="C2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D2" s="1">
         <v>46260</v>
@@ -1664,7 +1715,7 @@
         <v>2800672319</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D3" s="1">
         <v>45972</v>
@@ -1675,7 +1726,7 @@
         <v>1125525865</v>
       </c>
       <c r="C4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D4" s="1">
         <v>46296</v>
@@ -1686,7 +1737,7 @@
         <v>8104375203</v>
       </c>
       <c r="C5" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D5" s="1">
         <v>46128</v>
@@ -1697,7 +1748,7 @@
         <v>6724421141</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D6" s="1">
         <v>46276</v>
@@ -1708,7 +1759,7 @@
         <v>3428511303</v>
       </c>
       <c r="C7" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -1716,7 +1767,7 @@
         <v>7373366639</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D8" s="1">
         <v>46016</v>
@@ -1727,7 +1778,7 @@
         <v>6350095935</v>
       </c>
       <c r="C9" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D9" s="1">
         <v>46067</v>
@@ -1738,7 +1789,7 @@
         <v>3141284892</v>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D10" s="1">
         <v>46207</v>
@@ -1987,10 +2038,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B1" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -2048,16 +2099,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B1" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C1" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="D1" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -2065,7 +2116,7 @@
         <v>906296</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="C2" s="1">
         <v>46023</v>
@@ -2079,7 +2130,7 @@
         <v>814590</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -2087,7 +2138,7 @@
         <v>909166</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="C4" s="1">
         <v>44136</v>

</xml_diff>